<commit_message>
feat: Align Remision Folio to official format E0125 across database, UI and PDF generator
</commit_message>
<xml_diff>
--- a/data/sync_databases/BD_Datos_Generales_Remision.xlsx
+++ b/data/sync_databases/BD_Datos_Generales_Remision.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="674" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="674" uniqueCount="291">
   <si>
     <t>ID_Remision</t>
   </si>
@@ -337,9 +337,6 @@
     <t>E0125</t>
   </si>
   <si>
-    <t>REM-2608-054</t>
-  </si>
-  <si>
     <t>08/06/2026</t>
   </si>
   <si>
@@ -529,9 +526,6 @@
     <t>25/08/2026</t>
   </si>
   <si>
-    <t>2026-08-25 14:30:00</t>
-  </si>
-  <si>
     <t>Luis Quintana</t>
   </si>
   <si>
@@ -886,7 +880,7 @@
     <t>['TPM-0510', 'TPM-0509', 'TPM-0507', 'TPM-0493', 'TPM-0494', 'TPM-0495', 'TPM-0496', 'TPM-0504']</t>
   </si>
   <si>
-    <t>TPM-0511, TPM-0512, TPM-0513</t>
+    <t>['TPM-0511', 'TPM-0512', 'TPM-0513']</t>
   </si>
   <si>
     <t>TRANSPORTE INTERNO</t>
@@ -1267,22 +1261,22 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E2" t="s">
+        <v>176</v>
+      </c>
+      <c r="F2" t="s">
         <v>178</v>
       </c>
-      <c r="F2" t="s">
-        <v>180</v>
-      </c>
       <c r="G2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1293,22 +1287,22 @@
         <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F3" t="s">
         <v>178</v>
       </c>
-      <c r="F3" t="s">
-        <v>180</v>
-      </c>
       <c r="G3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1319,22 +1313,22 @@
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E4" t="s">
+        <v>176</v>
+      </c>
+      <c r="F4" t="s">
         <v>178</v>
       </c>
-      <c r="F4" t="s">
-        <v>180</v>
-      </c>
       <c r="G4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H4" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1345,22 +1339,22 @@
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E5" t="s">
+        <v>176</v>
+      </c>
+      <c r="F5" t="s">
         <v>178</v>
       </c>
-      <c r="F5" t="s">
-        <v>180</v>
-      </c>
       <c r="G5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1371,22 +1365,22 @@
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F6" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G6" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -1397,22 +1391,22 @@
         <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E7" t="s">
+        <v>176</v>
+      </c>
+      <c r="F7" t="s">
         <v>178</v>
       </c>
-      <c r="F7" t="s">
-        <v>180</v>
-      </c>
       <c r="G7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -1423,22 +1417,22 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E8" t="s">
+        <v>176</v>
+      </c>
+      <c r="F8" t="s">
         <v>178</v>
       </c>
-      <c r="F8" t="s">
-        <v>180</v>
-      </c>
       <c r="G8" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1449,22 +1443,22 @@
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E9" t="s">
+        <v>176</v>
+      </c>
+      <c r="F9" t="s">
         <v>178</v>
       </c>
-      <c r="F9" t="s">
-        <v>180</v>
-      </c>
       <c r="G9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -1475,22 +1469,22 @@
         <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D10" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E10" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F10" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G10" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H10" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -1501,22 +1495,22 @@
         <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D11" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E11" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F11" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G11" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H11" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -1527,22 +1521,22 @@
         <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D12" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E12" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G12" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1553,22 +1547,22 @@
         <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D13" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E13" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F13" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G13" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H13" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -1579,22 +1573,22 @@
         <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D14" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E14" t="s">
+        <v>176</v>
+      </c>
+      <c r="F14" t="s">
         <v>178</v>
       </c>
-      <c r="F14" t="s">
-        <v>180</v>
-      </c>
       <c r="G14" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H14" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1605,22 +1599,22 @@
         <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D15" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E15" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F15" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G15" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H15" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1631,19 +1625,19 @@
         <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D16" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F16" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G16" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H16" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1654,19 +1648,19 @@
         <v>25</v>
       </c>
       <c r="C17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D17" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F17" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G17" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H17" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1677,19 +1671,19 @@
         <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D18" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F18" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G18" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H18" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1700,19 +1694,19 @@
         <v>27</v>
       </c>
       <c r="C19" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D19" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F19" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G19" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H19" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1723,19 +1717,19 @@
         <v>28</v>
       </c>
       <c r="C20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D20" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F20" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G20" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H20" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1746,19 +1740,19 @@
         <v>29</v>
       </c>
       <c r="C21" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D21" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F21" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G21" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H21" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1769,19 +1763,19 @@
         <v>30</v>
       </c>
       <c r="C22" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D22" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F22" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G22" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H22" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1792,19 +1786,19 @@
         <v>31</v>
       </c>
       <c r="C23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D23" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F23" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H23" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1815,19 +1809,19 @@
         <v>32</v>
       </c>
       <c r="C24" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D24" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F24" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G24" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H24" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1838,19 +1832,19 @@
         <v>33</v>
       </c>
       <c r="C25" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D25" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F25" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G25" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H25" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1861,19 +1855,19 @@
         <v>34</v>
       </c>
       <c r="C26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D26" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F26" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G26" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H26" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1884,19 +1878,19 @@
         <v>35</v>
       </c>
       <c r="C27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D27" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F27" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G27" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H27" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1907,19 +1901,19 @@
         <v>36</v>
       </c>
       <c r="C28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D28" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F28" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G28" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H28" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1930,19 +1924,19 @@
         <v>37</v>
       </c>
       <c r="C29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D29" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F29" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G29" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H29" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1953,19 +1947,19 @@
         <v>38</v>
       </c>
       <c r="C30" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D30" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F30" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G30" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H30" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1976,19 +1970,19 @@
         <v>39</v>
       </c>
       <c r="C31" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D31" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F31" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G31" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H31" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1999,19 +1993,19 @@
         <v>40</v>
       </c>
       <c r="C32" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D32" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F32" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G32" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H32" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -2022,19 +2016,19 @@
         <v>41</v>
       </c>
       <c r="C33" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D33" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F33" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G33" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H33" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2045,19 +2039,19 @@
         <v>42</v>
       </c>
       <c r="C34" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D34" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F34" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G34" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H34" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2068,19 +2062,19 @@
         <v>43</v>
       </c>
       <c r="C35" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D35" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F35" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G35" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H35" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2091,19 +2085,19 @@
         <v>44</v>
       </c>
       <c r="C36" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D36" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F36" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G36" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H36" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2114,19 +2108,19 @@
         <v>45</v>
       </c>
       <c r="C37" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D37" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F37" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G37" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H37" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2137,19 +2131,19 @@
         <v>46</v>
       </c>
       <c r="C38" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D38" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F38" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G38" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H38" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2160,19 +2154,19 @@
         <v>47</v>
       </c>
       <c r="C39" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D39" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F39" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G39" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H39" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -2183,22 +2177,22 @@
         <v>48</v>
       </c>
       <c r="C40" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D40" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E40" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F40" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G40" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H40" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2209,22 +2203,22 @@
         <v>49</v>
       </c>
       <c r="C41" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D41" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E41" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F41" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G41" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H41" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -2235,22 +2229,22 @@
         <v>50</v>
       </c>
       <c r="C42" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D42" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E42" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F42" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G42" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H42" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2261,22 +2255,22 @@
         <v>51</v>
       </c>
       <c r="C43" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D43" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E43" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F43" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G43" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H43" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2287,22 +2281,22 @@
         <v>52</v>
       </c>
       <c r="C44" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D44" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E44" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F44" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G44" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H44" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2313,22 +2307,22 @@
         <v>53</v>
       </c>
       <c r="C45" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D45" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E45" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F45" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G45" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H45" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2339,22 +2333,22 @@
         <v>54</v>
       </c>
       <c r="C46" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D46" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E46" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F46" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G46" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H46" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -2365,22 +2359,22 @@
         <v>55</v>
       </c>
       <c r="C47" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D47" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E47" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F47" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G47" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H47" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2391,22 +2385,22 @@
         <v>56</v>
       </c>
       <c r="C48" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D48" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E48" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F48" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G48" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H48" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -2417,22 +2411,22 @@
         <v>57</v>
       </c>
       <c r="C49" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D49" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E49" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F49" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G49" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H49" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -2443,22 +2437,22 @@
         <v>58</v>
       </c>
       <c r="C50" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D50" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E50" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F50" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G50" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H50" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2469,22 +2463,22 @@
         <v>59</v>
       </c>
       <c r="C51" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D51" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E51" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F51" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G51" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H51" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2495,22 +2489,22 @@
         <v>60</v>
       </c>
       <c r="C52" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D52" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E52" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F52" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G52" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H52" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -2521,22 +2515,22 @@
         <v>61</v>
       </c>
       <c r="C53" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D53" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E53" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F53" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G53" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H53" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2547,22 +2541,22 @@
         <v>62</v>
       </c>
       <c r="C54" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D54" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E54" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F54" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G54" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H54" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2573,22 +2567,22 @@
         <v>63</v>
       </c>
       <c r="C55" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D55" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E55" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F55" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G55" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H55" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2599,22 +2593,22 @@
         <v>64</v>
       </c>
       <c r="C56" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D56" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E56" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F56" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G56" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H56" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -2625,22 +2619,22 @@
         <v>65</v>
       </c>
       <c r="C57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D57" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E57" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F57" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G57" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H57" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2651,22 +2645,22 @@
         <v>66</v>
       </c>
       <c r="C58" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D58" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E58" t="s">
+        <v>176</v>
+      </c>
+      <c r="F58" t="s">
         <v>178</v>
       </c>
-      <c r="F58" t="s">
-        <v>180</v>
-      </c>
       <c r="G58" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H58" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2677,22 +2671,22 @@
         <v>67</v>
       </c>
       <c r="C59" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D59" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E59" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F59" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G59" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H59" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2703,22 +2697,22 @@
         <v>68</v>
       </c>
       <c r="C60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D60" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E60" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F60" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G60" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H60" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -2729,22 +2723,22 @@
         <v>69</v>
       </c>
       <c r="C61" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D61" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E61" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F61" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G61" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H61" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -2755,22 +2749,22 @@
         <v>70</v>
       </c>
       <c r="C62" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D62" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E62" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F62" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G62" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H62" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -2781,22 +2775,22 @@
         <v>71</v>
       </c>
       <c r="C63" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D63" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E63" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F63" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G63" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H63" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -2807,22 +2801,22 @@
         <v>72</v>
       </c>
       <c r="C64" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D64" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E64" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F64" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G64" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H64" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -2833,22 +2827,22 @@
         <v>73</v>
       </c>
       <c r="C65" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D65" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E65" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F65" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G65" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H65" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -2859,22 +2853,22 @@
         <v>74</v>
       </c>
       <c r="C66" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D66" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E66" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F66" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G66" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H66" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -2885,22 +2879,22 @@
         <v>75</v>
       </c>
       <c r="C67" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D67" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E67" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F67" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G67" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H67" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -2911,22 +2905,22 @@
         <v>76</v>
       </c>
       <c r="C68" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D68" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E68" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F68" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G68" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H68" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -2937,22 +2931,22 @@
         <v>77</v>
       </c>
       <c r="C69" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D69" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E69" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F69" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G69" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H69" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -2963,22 +2957,22 @@
         <v>78</v>
       </c>
       <c r="C70" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D70" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E70" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F70" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G70" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H70" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -2989,22 +2983,22 @@
         <v>79</v>
       </c>
       <c r="C71" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D71" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E71" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F71" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G71" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H71" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -3015,22 +3009,22 @@
         <v>80</v>
       </c>
       <c r="C72" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D72" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E72" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F72" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G72" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H72" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -3041,22 +3035,22 @@
         <v>81</v>
       </c>
       <c r="C73" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D73" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E73" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F73" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G73" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H73" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -3067,22 +3061,22 @@
         <v>82</v>
       </c>
       <c r="C74" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D74" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E74" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F74" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G74" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H74" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -3093,22 +3087,22 @@
         <v>83</v>
       </c>
       <c r="C75" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D75" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E75" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F75" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G75" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H75" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -3119,22 +3113,22 @@
         <v>84</v>
       </c>
       <c r="C76" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D76" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E76" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F76" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G76" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H76" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -3145,22 +3139,22 @@
         <v>85</v>
       </c>
       <c r="C77" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D77" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E77" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F77" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G77" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H77" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -3171,22 +3165,22 @@
         <v>86</v>
       </c>
       <c r="C78" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D78" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E78" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F78" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G78" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H78" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -3197,22 +3191,22 @@
         <v>87</v>
       </c>
       <c r="C79" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D79" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E79" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F79" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G79" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H79" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -3223,22 +3217,22 @@
         <v>88</v>
       </c>
       <c r="C80" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D80" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E80" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F80" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G80" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H80" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="81" spans="1:8">
@@ -3249,22 +3243,22 @@
         <v>89</v>
       </c>
       <c r="C81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D81" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E81" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F81" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G81" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H81" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -3275,22 +3269,22 @@
         <v>90</v>
       </c>
       <c r="C82" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D82" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E82" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F82" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G82" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H82" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -3301,22 +3295,22 @@
         <v>91</v>
       </c>
       <c r="C83" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D83" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E83" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F83" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G83" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H83" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -3327,22 +3321,22 @@
         <v>92</v>
       </c>
       <c r="C84" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D84" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E84" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F84" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G84" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H84" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -3353,22 +3347,22 @@
         <v>93</v>
       </c>
       <c r="C85" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D85" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E85" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F85" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G85" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H85" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -3379,22 +3373,22 @@
         <v>94</v>
       </c>
       <c r="C86" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D86" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E86" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F86" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G86" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H86" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="87" spans="1:8">
@@ -3405,22 +3399,22 @@
         <v>95</v>
       </c>
       <c r="C87" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D87" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E87" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F87" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G87" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H87" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -3431,22 +3425,22 @@
         <v>96</v>
       </c>
       <c r="C88" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D88" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E88" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F88" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G88" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H88" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -3457,22 +3451,22 @@
         <v>97</v>
       </c>
       <c r="C89" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D89" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E89" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F89" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G89" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H89" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -3483,22 +3477,22 @@
         <v>98</v>
       </c>
       <c r="C90" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D90" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E90" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F90" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G90" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H90" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -3509,22 +3503,22 @@
         <v>99</v>
       </c>
       <c r="C91" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D91" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E91" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F91" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G91" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H91" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -3535,22 +3529,22 @@
         <v>100</v>
       </c>
       <c r="C92" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D92" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E92" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F92" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G92" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H92" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -3561,22 +3555,22 @@
         <v>101</v>
       </c>
       <c r="C93" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D93" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E93" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F93" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G93" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H93" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -3587,22 +3581,22 @@
         <v>102</v>
       </c>
       <c r="C94" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D94" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E94" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F94" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G94" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H94" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -3613,22 +3607,22 @@
         <v>103</v>
       </c>
       <c r="C95" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D95" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E95" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F95" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G95" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H95" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -3639,22 +3633,22 @@
         <v>104</v>
       </c>
       <c r="C96" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E96" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F96" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G96" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H96" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="97" spans="1:10">
@@ -3665,22 +3659,22 @@
         <v>105</v>
       </c>
       <c r="C97" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D97" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E97" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F97" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G97" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H97" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="98" spans="1:10">
@@ -3691,22 +3685,22 @@
         <v>106</v>
       </c>
       <c r="C98" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D98" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E98" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F98" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G98" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H98" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="99" spans="1:10">
@@ -3714,31 +3708,31 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C99" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D99" t="s">
+        <v>175</v>
+      </c>
+      <c r="E99" t="s">
         <v>177</v>
       </c>
-      <c r="E99" t="s">
+      <c r="F99" t="s">
         <v>179</v>
       </c>
-      <c r="F99" t="s">
-        <v>181</v>
-      </c>
       <c r="G99" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="H99" t="s">
+        <v>288</v>
+      </c>
+      <c r="I99" t="s">
+        <v>289</v>
+      </c>
+      <c r="J99" t="s">
         <v>290</v>
-      </c>
-      <c r="I99" t="s">
-        <v>291</v>
-      </c>
-      <c r="J99" t="s">
-        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>